<commit_message>
Fix import template sample data
</commit_message>
<xml_diff>
--- a/sample-data/Mau_Import_HoDan.xlsx
+++ b/sample-data/Mau_Import_HoDan.xlsx
@@ -133,6 +133,147 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="2">
+        <is>
+          <t>HD001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="2">
+        <is>
+          <t>Nguyễn Văn An</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="2">
+        <is>
+          <t>Thôn 9, Xã Minh Châu</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
+          <t>0912345678</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr" s="2">
+        <is>
+          <t>THON09</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="2">
+        <is>
+          <t>Ho binh thuong</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr" s="2">
+        <is>
+          <t>Khong</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr" s="2">
+        <is>
+          <t>Khong</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr" s="2">
+        <is>
+          <t>Hộ mẫu có nhiều thế hệ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="2">
+        <is>
+          <t>HD002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t>Trần Thị Bình</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t>Thôn 9, Xã Minh Châu</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="2">
+        <is>
+          <t>THON09</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="2">
+        <is>
+          <t>Ho can ngheo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="2">
+        <is>
+          <t>Khong</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr" s="2">
+        <is>
+          <t>Co</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr" s="2">
+        <is>
+          <t>Hộ mẫu cận nghèo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="2">
+        <is>
+          <t>HD003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t>Lê Văn Cường</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>Thôn 9, Xã Minh Châu</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>0901122334</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>THON09</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t>Ho chinh sach</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="2">
+        <is>
+          <t>Khong</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="2">
+        <is>
+          <t>Khong</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr" s="2">
+        <is>
+          <t>Hộ mẫu chính sách</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -212,17 +353,29 @@
       </c>
       <c r="B6" t="inlineStr" s="2">
         <is>
-          <t>Nhap Co, Khong, 1, 0, X. Neu bo trong thi hieu la Khong, rieng BHYT bo trong mac dinh la Co.</t>
+          <t>Nhap Co, Khong, 1, 0, X. Neu bo trong thi hieu la Khong. BHYT chi mac dinh Co theo cot Nghe nghiep khi la Hoc sinh hoac Nguoi cao tuoi (70+).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="2">
         <is>
+          <t>Quan he voi chu ho</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t>Co the de trong. Sau import he thong chi tu suy luan trong cung ho khi du du lieu bo/me/chu ho va khong ghi de gia tri da nhap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
           <t>Ho co cong/khuyet tat</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr" s="2">
+      <c r="B8" t="inlineStr" s="2">
         <is>
           <t>Khong nhap o mau ho dan. He thong tu suy ra tu cac cot chinh sach cua nhan khau trong ho.</t>
         </is>

</xml_diff>